<commit_message>
fix: fixed dumb mistake
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -641,7 +641,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H2" s="3" t="n"/>
@@ -725,7 +725,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H4" s="3" t="n"/>
@@ -769,7 +769,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>max 500 chars</t>
+          <t>max 500 characters</t>
         </is>
       </c>
       <c r="H5" s="3" t="n"/>
@@ -893,7 +893,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H8" s="3" t="n"/>
@@ -937,7 +937,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H9" s="3" t="n"/>
@@ -981,7 +981,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H10" s="3" t="n"/>
@@ -1025,7 +1025,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H11" s="3" t="n"/>
@@ -1149,7 +1149,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H14" s="3" t="n"/>
@@ -1313,7 +1313,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H18" s="3" t="n"/>
@@ -1397,7 +1397,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H20" s="3" t="n"/>
@@ -1481,7 +1481,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H22" s="3" t="n"/>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H27" s="3" t="n"/>
@@ -1733,7 +1733,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H28" s="3" t="n"/>
@@ -1777,7 +1777,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H29" s="3" t="n"/>
@@ -1821,7 +1821,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H30" s="3" t="n"/>
@@ -1865,7 +1865,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H31" s="3" t="n"/>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H32" s="3" t="n"/>
@@ -1953,7 +1953,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H33" s="3" t="n"/>
@@ -1997,7 +1997,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H34" s="3" t="n"/>
@@ -2041,7 +2041,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H35" s="3" t="n"/>
@@ -2085,7 +2085,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H36" s="3" t="n"/>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>max 100 chars</t>
+          <t>max 100 characters</t>
         </is>
       </c>
       <c r="H37" s="3" t="n"/>
@@ -2825,7 +2825,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>max 500 chars</t>
+          <t>max 500 characters</t>
         </is>
       </c>
       <c r="H54" s="3" t="n"/>
@@ -2949,7 +2949,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>max 100 chars</t>
+          <t>max 100 characters</t>
         </is>
       </c>
       <c r="H57" s="3" t="n"/>
@@ -3329,7 +3329,7 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>max 500 chars</t>
+          <t>max 500 characters</t>
         </is>
       </c>
       <c r="H66" s="3" t="n"/>
@@ -4193,7 +4193,7 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H86" s="3" t="n"/>
@@ -4237,7 +4237,7 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H87" s="3" t="n"/>
@@ -4281,7 +4281,7 @@
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H88" s="3" t="n"/>
@@ -4325,7 +4325,7 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H89" s="3" t="n"/>
@@ -4369,7 +4369,7 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H90" s="3" t="n"/>
@@ -4413,7 +4413,7 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H91" s="3" t="n"/>
@@ -4457,7 +4457,7 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H92" s="3" t="n"/>
@@ -4501,7 +4501,7 @@
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H93" s="3" t="n"/>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H94" s="3" t="n"/>
@@ -7028,54 +7028,54 @@
       <c r="C4" s="3" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>max 200 chars</t>
+          <t>max 200 characters</t>
         </is>
       </c>
       <c r="P4" s="3" t="inlineStr"/>

</xml_diff>

<commit_message>
feat: don't remember but many great things i am sure
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -7165,7 +7165,11 @@
           <t>Requirements</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n"/>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Recommended</t>
@@ -17382,7 +17386,11 @@
           <t>Requirements</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n"/>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Required</t>
@@ -55564,7 +55572,7 @@
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
     <col width="37" customWidth="1" min="5" max="5"/>
     <col width="38" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
@@ -55605,7 +55613,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>LCA stages</t>
+          <t>LCA stage or module</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -55849,7 +55857,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>LCAStages</t>
+          <t>LCAStageOrModule</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -56107,7 +56115,11 @@
           <t>Requirements</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n"/>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
       <c r="C6" s="7" t="n"/>
       <c r="D6" s="6" t="inlineStr">
         <is>
@@ -56240,7 +56252,7 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>lca_stages</t>
+          <t>lca_stage_or_module</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
@@ -58973,7 +58985,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="D9:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>TypeDefinitions!$Z$2:$Z$24</formula1>
+      <formula1>TypeDefinitions!$Z$2:$Z$25</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -58991,7 +59003,7 @@
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
     <col width="27" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="28.5" customWidth="1" min="6" max="6"/>
@@ -59000,7 +59012,7 @@
     <col width="54" customWidth="1" min="9" max="9"/>
     <col width="42" customWidth="1" min="10" max="10"/>
     <col width="52.5" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
     <col width="24" customWidth="1" min="13" max="13"/>
     <col width="31.5" customWidth="1" min="14" max="14"/>
     <col width="37.5" customWidth="1" min="15" max="15"/>
@@ -59014,7 +59026,7 @@
     <col width="27" customWidth="1" min="23" max="23"/>
     <col width="57" customWidth="1" min="24" max="24"/>
     <col width="46.5" customWidth="1" min="25" max="25"/>
-    <col width="16.5" customWidth="1" min="26" max="26"/>
+    <col width="27" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -59145,7 +59157,7 @@
       </c>
       <c r="Z1" s="12" t="inlineStr">
         <is>
-          <t>LCAStages</t>
+          <t>LCAStageOrModule</t>
         </is>
       </c>
     </row>
@@ -60504,7 +60516,7 @@
       </c>
       <c r="Z23" t="inlineStr">
         <is>
-          <t>D1 Reuse, recovery, and recycling potential</t>
+          <t>D Benefits and loads beyond the system boundary</t>
         </is>
       </c>
     </row>
@@ -60526,7 +60538,7 @@
       </c>
       <c r="Z24" t="inlineStr">
         <is>
-          <t>D2 Net benefits beyond the system boundary</t>
+          <t>D1 Reuse, recovery, and recycling potential</t>
         </is>
       </c>
     </row>
@@ -60544,6 +60556,11 @@
       <c r="X25" t="inlineStr">
         <is>
           <t>4.1 General FF&amp;E</t>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>D2 Net benefits beyond the system boundary</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: update templates with default value columns
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -6478,7 +6478,7 @@
       <formula1>1900-01-01</formula1>
     </dataValidation>
     <dataValidation sqref="J38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>TypeDefinitions!$F$2:$F$10</formula1>
+      <formula1>TypeDefinitions!$F$2:$F$15</formula1>
     </dataValidation>
     <dataValidation sqref="J40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>TypeDefinitions!$G$2:$G$7</formula1>
@@ -6672,31 +6672,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V109"/>
+  <dimension ref="A1:S109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="27" customWidth="1" min="5" max="5"/>
-    <col width="27" customWidth="1" min="6" max="6"/>
-    <col width="27" customWidth="1" min="7" max="7"/>
-    <col width="27" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="44" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
-    <col width="43" customWidth="1" min="12" max="12"/>
-    <col width="26" customWidth="1" min="13" max="13"/>
-    <col width="36" customWidth="1" min="14" max="14"/>
-    <col width="31" customWidth="1" min="15" max="15"/>
-    <col width="31" customWidth="1" min="16" max="16"/>
-    <col width="27" customWidth="1" min="17" max="17"/>
-    <col width="27" customWidth="1" min="18" max="18"/>
-    <col width="26" customWidth="1" min="19" max="19"/>
-    <col width="30" customWidth="1" min="20" max="20"/>
-    <col width="25" customWidth="1" min="21" max="21"/>
-    <col width="15" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="43" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="11" max="11"/>
+    <col width="31" customWidth="1" min="12" max="12"/>
+    <col width="31" customWidth="1" min="13" max="13"/>
+    <col width="27" customWidth="1" min="14" max="14"/>
+    <col width="27" customWidth="1" min="15" max="15"/>
+    <col width="26" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="17" max="17"/>
+    <col width="25" customWidth="1" min="18" max="18"/>
+    <col width="15" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6722,90 +6719,75 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Element Class (Tier 1)</t>
+          <t>Element Class</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Element Class (Tier 2)</t>
+          <t>Element Class Description</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Element Class (Tier 3)</t>
+          <t>OpenBDF Building Element Classification</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Element Class (Tier 4)</t>
+          <t>Element Name (or ID)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Element Class Description</t>
+          <t>OpenBDF Common Material Classification</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>OpenBDF Building Element Classification</t>
+          <t>Material Name (or ID)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Element Name (or ID)</t>
+          <t>Material Name from EPD database</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>OpenBDF Common Material Classification</t>
+          <t>Material EPD Database Name</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Material Name (or ID)</t>
+          <t>Material EPD Database Link</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Material Name from EPD database</t>
+          <t>Material Quantity (m3)</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Material EPD Database Name</t>
+          <t>Material Quantity (m2)</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Material EPD Database Link</t>
+          <t>Material Quantity (m)</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Material Quantity (m3)</t>
+          <t>Material Quantity (count)</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Material Quantity (m2)</t>
+          <t>Material Weight (kg)</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Material Quantity (m)</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Material Quantity (count)</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>Material Weight (kg)</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Density</t>
         </is>
@@ -6834,90 +6816,75 @@
       </c>
       <c r="E2" s="10" t="inlineStr">
         <is>
-          <t>Primary (top-level) hierarchical category of the custom or national building element classification.</t>
+          <t>Hierarchical category of the custom or national building element classification.</t>
         </is>
       </c>
       <c r="F2" s="10" t="inlineStr">
         <is>
-          <t>Secondary hierarchical category of the custom or national building element classification.</t>
+          <t>The Description of the custom or national element class.</t>
         </is>
       </c>
       <c r="G2" s="10" t="inlineStr">
         <is>
-          <t>The tertiary hierarchical category of the custom or national building element classification.</t>
+          <t>The highest applicable tier of the building element within the standardized openBDF framework.</t>
         </is>
       </c>
       <c r="H2" s="10" t="inlineStr">
         <is>
-          <t>The quaternary (lowest-level) hierarchical category of the custom or national building element classification.</t>
+          <t>The specific, user-defined identifier for the building element.</t>
         </is>
       </c>
       <c r="I2" s="10" t="inlineStr">
         <is>
-          <t>The Description of the custom or national element class.</t>
-        </is>
-      </c>
-      <c r="J2" s="10" t="inlineStr">
-        <is>
-          <t>The highest applicable tier of the building element within the standardized openBDF framework.</t>
+          <t>The corresponding material classification from the standardized openBDF taxonomy.</t>
+        </is>
+      </c>
+      <c r="J2" s="9" t="inlineStr">
+        <is>
+          <t>The specific, user-defined identifier for the material.</t>
         </is>
       </c>
       <c r="K2" s="10" t="inlineStr">
         <is>
-          <t>The specific, user-defined identifier for the building element.</t>
+          <t>The precise material designation as cataloged in the associated Environmental Product Declaration (EPD) database.</t>
         </is>
       </c>
       <c r="L2" s="10" t="inlineStr">
         <is>
-          <t>The corresponding material classification from the standardized openBDF taxonomy.</t>
-        </is>
-      </c>
-      <c r="M2" s="9" t="inlineStr">
-        <is>
-          <t>The specific, user-defined identifier for the material.</t>
+          <t>The nomenclature of the specific Environmental Product Declaration (EPD) dataset used.</t>
+        </is>
+      </c>
+      <c r="M2" s="10" t="inlineStr">
+        <is>
+          <t>The URL of the specific Environmental Product Declaration (EPD) dataset used.</t>
         </is>
       </c>
       <c r="N2" s="10" t="inlineStr">
         <is>
-          <t>The precise material designation as cataloged in the associated Environmental Product Declaration (EPD) database.</t>
+          <t>The measured scalar amount (volume) of the custom material.</t>
         </is>
       </c>
       <c r="O2" s="10" t="inlineStr">
         <is>
-          <t>The nomenclature of the specific Environmental Product Declaration (EPD) dataset used.</t>
+          <t>The measured scalar amount (area) of the custom material.</t>
         </is>
       </c>
       <c r="P2" s="10" t="inlineStr">
         <is>
-          <t>The URL of the specific Environmental Product Declaration (EPD) dataset used.</t>
+          <t>The measured scalar amount (length) of the custom material.</t>
         </is>
       </c>
       <c r="Q2" s="10" t="inlineStr">
         <is>
-          <t>The measured scalar amount (volume) of the custom material.</t>
+          <t>The measured scalar amount (count) of the custom material.</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
         <is>
-          <t>The measured scalar amount (area) of the custom material.</t>
+          <t>The absolute physical mass of the custom material.</t>
         </is>
       </c>
       <c r="S2" s="10" t="inlineStr">
-        <is>
-          <t>The measured scalar amount (length) of the custom material.</t>
-        </is>
-      </c>
-      <c r="T2" s="10" t="inlineStr">
-        <is>
-          <t>The measured scalar amount (count) of the custom material.</t>
-        </is>
-      </c>
-      <c r="U2" s="10" t="inlineStr">
-        <is>
-          <t>The absolute physical mass of the custom material.</t>
-        </is>
-      </c>
-      <c r="V2" s="10" t="inlineStr">
         <is>
           <t>The mass per unit volume of the custom material.</t>
         </is>
@@ -6956,34 +6923,34 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>OpenBDFBuildingElementClassification</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>string</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>OpenBDFMaterialClassification</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>OpenBDFBuildingElementClassification</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>OpenBDFMaterialClassification</t>
-        </is>
-      </c>
       <c r="M3" t="inlineStr">
         <is>
           <t>string</t>
@@ -6991,17 +6958,17 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>Decimal</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>Decimal</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>Decimal</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -7015,21 +6982,6 @@
         </is>
       </c>
       <c r="S3" t="inlineStr">
-        <is>
-          <t>Decimal</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>Decimal</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Decimal</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
         <is>
           <t>Decimal</t>
         </is>
@@ -7058,54 +7010,39 @@
           <t>max 200 characters</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>max 200 characters</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>max 200 characters</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>max 200 characters</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>max 200 characters</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr">
         <is>
           <t>max 200 characters</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>max 200 characters</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>max 200 characters</t>
-        </is>
-      </c>
-      <c r="P4" s="2" t="inlineStr">
-        <is>
-          <t>max 200 characters</t>
-        </is>
-      </c>
+      <c r="N4" s="3" t="inlineStr"/>
+      <c r="O4" s="3" t="inlineStr"/>
+      <c r="P4" s="3" t="inlineStr"/>
       <c r="Q4" s="3" t="inlineStr"/>
       <c r="R4" s="3" t="inlineStr"/>
       <c r="S4" s="3" t="inlineStr"/>
-      <c r="T4" s="3" t="inlineStr"/>
-      <c r="U4" s="3" t="inlineStr"/>
-      <c r="V4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -7125,35 +7062,32 @@
       <c r="K5" s="3" t="n"/>
       <c r="L5" s="3" t="n"/>
       <c r="M5" s="3" t="n"/>
-      <c r="N5" s="3" t="n"/>
-      <c r="O5" s="3" t="n"/>
-      <c r="P5" s="3" t="n"/>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>#</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="S5" s="2" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="T5" s="2" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="U5" s="2" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="V5" s="2" t="inlineStr">
         <is>
           <t>kg/m3</t>
         </is>
@@ -7195,77 +7129,62 @@
           <t>Recommended</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="L6" s="4" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="M6" s="7" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="L6" s="7" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="M6" s="6" t="inlineStr">
+      <c r="O6" s="4" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="P6" s="4" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="Q6" s="4" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="R6" s="6" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="N6" s="4" t="inlineStr">
-        <is>
-          <t>Recommended</t>
-        </is>
-      </c>
-      <c r="O6" s="4" t="inlineStr">
-        <is>
-          <t>Recommended</t>
-        </is>
-      </c>
-      <c r="P6" s="7" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="Q6" s="4" t="inlineStr">
-        <is>
-          <t>Recommended</t>
-        </is>
-      </c>
-      <c r="R6" s="4" t="inlineStr">
-        <is>
-          <t>Recommended</t>
-        </is>
-      </c>
       <c r="S6" s="4" t="inlineStr">
-        <is>
-          <t>Recommended</t>
-        </is>
-      </c>
-      <c r="T6" s="4" t="inlineStr">
-        <is>
-          <t>Recommended</t>
-        </is>
-      </c>
-      <c r="U6" s="6" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="V6" s="4" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
@@ -7301,90 +7220,75 @@
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>bec_custom_tier1</t>
+          <t>bec_custom</t>
         </is>
       </c>
       <c r="F8" s="11" t="inlineStr">
         <is>
-          <t>bec_custom_tier2</t>
+          <t>bec_custom_description</t>
         </is>
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>bec_custom_tier3</t>
+          <t>bec_openbdf_selection</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>bec_custom_tier4</t>
+          <t>element_name_custom</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>bec_custom_description</t>
+          <t>openbdf_material_name</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr">
         <is>
-          <t>bec_openbdf_selection</t>
+          <t>material_name_custom</t>
         </is>
       </c>
       <c r="K8" s="11" t="inlineStr">
         <is>
-          <t>element_name_custom</t>
+          <t>material_name_database</t>
         </is>
       </c>
       <c r="L8" s="11" t="inlineStr">
         <is>
-          <t>openbdf_material_name</t>
+          <t>lca_dataset_name</t>
         </is>
       </c>
       <c r="M8" s="11" t="inlineStr">
         <is>
-          <t>material_name_custom</t>
+          <t>lca_dataset_link</t>
         </is>
       </c>
       <c r="N8" s="11" t="inlineStr">
         <is>
-          <t>material_name_database</t>
+          <t>custom_material_quantity_m3</t>
         </is>
       </c>
       <c r="O8" s="11" t="inlineStr">
         <is>
-          <t>lca_dataset_name</t>
+          <t>custom_material_quantity_m2</t>
         </is>
       </c>
       <c r="P8" s="11" t="inlineStr">
         <is>
-          <t>lca_dataset_link</t>
+          <t>custom_material_quantity_m</t>
         </is>
       </c>
       <c r="Q8" s="11" t="inlineStr">
         <is>
-          <t>custom_material_quantity_m3</t>
+          <t>custom_material_quantity_count</t>
         </is>
       </c>
       <c r="R8" s="11" t="inlineStr">
         <is>
-          <t>custom_material_quantity_m2</t>
+          <t>custom_material_weight_kg</t>
         </is>
       </c>
       <c r="S8" s="11" t="inlineStr">
-        <is>
-          <t>custom_material_quantity_m</t>
-        </is>
-      </c>
-      <c r="T8" s="11" t="inlineStr">
-        <is>
-          <t>custom_material_quantity_count</t>
-        </is>
-      </c>
-      <c r="U8" s="11" t="inlineStr">
-        <is>
-          <t>custom_material_weight_kg</t>
-        </is>
-      </c>
-      <c r="V8" s="11" t="inlineStr">
         <is>
           <t>custom_material_density</t>
         </is>
@@ -7410,9 +7314,6 @@
       <c r="Q9" s="5" t="n"/>
       <c r="R9" s="5" t="n"/>
       <c r="S9" s="5" t="n"/>
-      <c r="T9" s="5" t="n"/>
-      <c r="U9" s="5" t="n"/>
-      <c r="V9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n"/>
@@ -7434,9 +7335,6 @@
       <c r="Q10" s="5" t="n"/>
       <c r="R10" s="5" t="n"/>
       <c r="S10" s="5" t="n"/>
-      <c r="T10" s="5" t="n"/>
-      <c r="U10" s="5" t="n"/>
-      <c r="V10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n"/>
@@ -7458,9 +7356,6 @@
       <c r="Q11" s="5" t="n"/>
       <c r="R11" s="5" t="n"/>
       <c r="S11" s="5" t="n"/>
-      <c r="T11" s="5" t="n"/>
-      <c r="U11" s="5" t="n"/>
-      <c r="V11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n"/>
@@ -7482,9 +7377,6 @@
       <c r="Q12" s="5" t="n"/>
       <c r="R12" s="5" t="n"/>
       <c r="S12" s="5" t="n"/>
-      <c r="T12" s="5" t="n"/>
-      <c r="U12" s="5" t="n"/>
-      <c r="V12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n"/>
@@ -7506,9 +7398,6 @@
       <c r="Q13" s="5" t="n"/>
       <c r="R13" s="5" t="n"/>
       <c r="S13" s="5" t="n"/>
-      <c r="T13" s="5" t="n"/>
-      <c r="U13" s="5" t="n"/>
-      <c r="V13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n"/>
@@ -7530,9 +7419,6 @@
       <c r="Q14" s="5" t="n"/>
       <c r="R14" s="5" t="n"/>
       <c r="S14" s="5" t="n"/>
-      <c r="T14" s="5" t="n"/>
-      <c r="U14" s="5" t="n"/>
-      <c r="V14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n"/>
@@ -7554,9 +7440,6 @@
       <c r="Q15" s="5" t="n"/>
       <c r="R15" s="5" t="n"/>
       <c r="S15" s="5" t="n"/>
-      <c r="T15" s="5" t="n"/>
-      <c r="U15" s="5" t="n"/>
-      <c r="V15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n"/>
@@ -7578,9 +7461,6 @@
       <c r="Q16" s="5" t="n"/>
       <c r="R16" s="5" t="n"/>
       <c r="S16" s="5" t="n"/>
-      <c r="T16" s="5" t="n"/>
-      <c r="U16" s="5" t="n"/>
-      <c r="V16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n"/>
@@ -7602,9 +7482,6 @@
       <c r="Q17" s="5" t="n"/>
       <c r="R17" s="5" t="n"/>
       <c r="S17" s="5" t="n"/>
-      <c r="T17" s="5" t="n"/>
-      <c r="U17" s="5" t="n"/>
-      <c r="V17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n"/>
@@ -7626,9 +7503,6 @@
       <c r="Q18" s="5" t="n"/>
       <c r="R18" s="5" t="n"/>
       <c r="S18" s="5" t="n"/>
-      <c r="T18" s="5" t="n"/>
-      <c r="U18" s="5" t="n"/>
-      <c r="V18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n"/>
@@ -7650,9 +7524,6 @@
       <c r="Q19" s="5" t="n"/>
       <c r="R19" s="5" t="n"/>
       <c r="S19" s="5" t="n"/>
-      <c r="T19" s="5" t="n"/>
-      <c r="U19" s="5" t="n"/>
-      <c r="V19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n"/>
@@ -7674,9 +7545,6 @@
       <c r="Q20" s="5" t="n"/>
       <c r="R20" s="5" t="n"/>
       <c r="S20" s="5" t="n"/>
-      <c r="T20" s="5" t="n"/>
-      <c r="U20" s="5" t="n"/>
-      <c r="V20" s="5" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n"/>
@@ -7698,9 +7566,6 @@
       <c r="Q21" s="5" t="n"/>
       <c r="R21" s="5" t="n"/>
       <c r="S21" s="5" t="n"/>
-      <c r="T21" s="5" t="n"/>
-      <c r="U21" s="5" t="n"/>
-      <c r="V21" s="5" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n"/>
@@ -7722,9 +7587,6 @@
       <c r="Q22" s="5" t="n"/>
       <c r="R22" s="5" t="n"/>
       <c r="S22" s="5" t="n"/>
-      <c r="T22" s="5" t="n"/>
-      <c r="U22" s="5" t="n"/>
-      <c r="V22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n"/>
@@ -7746,9 +7608,6 @@
       <c r="Q23" s="5" t="n"/>
       <c r="R23" s="5" t="n"/>
       <c r="S23" s="5" t="n"/>
-      <c r="T23" s="5" t="n"/>
-      <c r="U23" s="5" t="n"/>
-      <c r="V23" s="5" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n"/>
@@ -7770,9 +7629,6 @@
       <c r="Q24" s="5" t="n"/>
       <c r="R24" s="5" t="n"/>
       <c r="S24" s="5" t="n"/>
-      <c r="T24" s="5" t="n"/>
-      <c r="U24" s="5" t="n"/>
-      <c r="V24" s="5" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n"/>
@@ -7794,9 +7650,6 @@
       <c r="Q25" s="5" t="n"/>
       <c r="R25" s="5" t="n"/>
       <c r="S25" s="5" t="n"/>
-      <c r="T25" s="5" t="n"/>
-      <c r="U25" s="5" t="n"/>
-      <c r="V25" s="5" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n"/>
@@ -7818,9 +7671,6 @@
       <c r="Q26" s="5" t="n"/>
       <c r="R26" s="5" t="n"/>
       <c r="S26" s="5" t="n"/>
-      <c r="T26" s="5" t="n"/>
-      <c r="U26" s="5" t="n"/>
-      <c r="V26" s="5" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n"/>
@@ -7842,9 +7692,6 @@
       <c r="Q27" s="5" t="n"/>
       <c r="R27" s="5" t="n"/>
       <c r="S27" s="5" t="n"/>
-      <c r="T27" s="5" t="n"/>
-      <c r="U27" s="5" t="n"/>
-      <c r="V27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n"/>
@@ -7866,9 +7713,6 @@
       <c r="Q28" s="5" t="n"/>
       <c r="R28" s="5" t="n"/>
       <c r="S28" s="5" t="n"/>
-      <c r="T28" s="5" t="n"/>
-      <c r="U28" s="5" t="n"/>
-      <c r="V28" s="5" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n"/>
@@ -7890,9 +7734,6 @@
       <c r="Q29" s="5" t="n"/>
       <c r="R29" s="5" t="n"/>
       <c r="S29" s="5" t="n"/>
-      <c r="T29" s="5" t="n"/>
-      <c r="U29" s="5" t="n"/>
-      <c r="V29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n"/>
@@ -7914,9 +7755,6 @@
       <c r="Q30" s="5" t="n"/>
       <c r="R30" s="5" t="n"/>
       <c r="S30" s="5" t="n"/>
-      <c r="T30" s="5" t="n"/>
-      <c r="U30" s="5" t="n"/>
-      <c r="V30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n"/>
@@ -7938,9 +7776,6 @@
       <c r="Q31" s="5" t="n"/>
       <c r="R31" s="5" t="n"/>
       <c r="S31" s="5" t="n"/>
-      <c r="T31" s="5" t="n"/>
-      <c r="U31" s="5" t="n"/>
-      <c r="V31" s="5" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n"/>
@@ -7962,9 +7797,6 @@
       <c r="Q32" s="5" t="n"/>
       <c r="R32" s="5" t="n"/>
       <c r="S32" s="5" t="n"/>
-      <c r="T32" s="5" t="n"/>
-      <c r="U32" s="5" t="n"/>
-      <c r="V32" s="5" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n"/>
@@ -7986,9 +7818,6 @@
       <c r="Q33" s="5" t="n"/>
       <c r="R33" s="5" t="n"/>
       <c r="S33" s="5" t="n"/>
-      <c r="T33" s="5" t="n"/>
-      <c r="U33" s="5" t="n"/>
-      <c r="V33" s="5" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n"/>
@@ -8010,9 +7839,6 @@
       <c r="Q34" s="5" t="n"/>
       <c r="R34" s="5" t="n"/>
       <c r="S34" s="5" t="n"/>
-      <c r="T34" s="5" t="n"/>
-      <c r="U34" s="5" t="n"/>
-      <c r="V34" s="5" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n"/>
@@ -8034,9 +7860,6 @@
       <c r="Q35" s="5" t="n"/>
       <c r="R35" s="5" t="n"/>
       <c r="S35" s="5" t="n"/>
-      <c r="T35" s="5" t="n"/>
-      <c r="U35" s="5" t="n"/>
-      <c r="V35" s="5" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n"/>
@@ -8058,9 +7881,6 @@
       <c r="Q36" s="5" t="n"/>
       <c r="R36" s="5" t="n"/>
       <c r="S36" s="5" t="n"/>
-      <c r="T36" s="5" t="n"/>
-      <c r="U36" s="5" t="n"/>
-      <c r="V36" s="5" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n"/>
@@ -8082,9 +7902,6 @@
       <c r="Q37" s="5" t="n"/>
       <c r="R37" s="5" t="n"/>
       <c r="S37" s="5" t="n"/>
-      <c r="T37" s="5" t="n"/>
-      <c r="U37" s="5" t="n"/>
-      <c r="V37" s="5" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n"/>
@@ -8106,9 +7923,6 @@
       <c r="Q38" s="5" t="n"/>
       <c r="R38" s="5" t="n"/>
       <c r="S38" s="5" t="n"/>
-      <c r="T38" s="5" t="n"/>
-      <c r="U38" s="5" t="n"/>
-      <c r="V38" s="5" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n"/>
@@ -8130,9 +7944,6 @@
       <c r="Q39" s="5" t="n"/>
       <c r="R39" s="5" t="n"/>
       <c r="S39" s="5" t="n"/>
-      <c r="T39" s="5" t="n"/>
-      <c r="U39" s="5" t="n"/>
-      <c r="V39" s="5" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n"/>
@@ -8154,9 +7965,6 @@
       <c r="Q40" s="5" t="n"/>
       <c r="R40" s="5" t="n"/>
       <c r="S40" s="5" t="n"/>
-      <c r="T40" s="5" t="n"/>
-      <c r="U40" s="5" t="n"/>
-      <c r="V40" s="5" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n"/>
@@ -8178,9 +7986,6 @@
       <c r="Q41" s="5" t="n"/>
       <c r="R41" s="5" t="n"/>
       <c r="S41" s="5" t="n"/>
-      <c r="T41" s="5" t="n"/>
-      <c r="U41" s="5" t="n"/>
-      <c r="V41" s="5" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n"/>
@@ -8202,9 +8007,6 @@
       <c r="Q42" s="5" t="n"/>
       <c r="R42" s="5" t="n"/>
       <c r="S42" s="5" t="n"/>
-      <c r="T42" s="5" t="n"/>
-      <c r="U42" s="5" t="n"/>
-      <c r="V42" s="5" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n"/>
@@ -8226,9 +8028,6 @@
       <c r="Q43" s="5" t="n"/>
       <c r="R43" s="5" t="n"/>
       <c r="S43" s="5" t="n"/>
-      <c r="T43" s="5" t="n"/>
-      <c r="U43" s="5" t="n"/>
-      <c r="V43" s="5" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n"/>
@@ -8250,9 +8049,6 @@
       <c r="Q44" s="5" t="n"/>
       <c r="R44" s="5" t="n"/>
       <c r="S44" s="5" t="n"/>
-      <c r="T44" s="5" t="n"/>
-      <c r="U44" s="5" t="n"/>
-      <c r="V44" s="5" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="n"/>
@@ -8274,9 +8070,6 @@
       <c r="Q45" s="5" t="n"/>
       <c r="R45" s="5" t="n"/>
       <c r="S45" s="5" t="n"/>
-      <c r="T45" s="5" t="n"/>
-      <c r="U45" s="5" t="n"/>
-      <c r="V45" s="5" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n"/>
@@ -8298,9 +8091,6 @@
       <c r="Q46" s="5" t="n"/>
       <c r="R46" s="5" t="n"/>
       <c r="S46" s="5" t="n"/>
-      <c r="T46" s="5" t="n"/>
-      <c r="U46" s="5" t="n"/>
-      <c r="V46" s="5" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n"/>
@@ -8322,9 +8112,6 @@
       <c r="Q47" s="5" t="n"/>
       <c r="R47" s="5" t="n"/>
       <c r="S47" s="5" t="n"/>
-      <c r="T47" s="5" t="n"/>
-      <c r="U47" s="5" t="n"/>
-      <c r="V47" s="5" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n"/>
@@ -8346,9 +8133,6 @@
       <c r="Q48" s="5" t="n"/>
       <c r="R48" s="5" t="n"/>
       <c r="S48" s="5" t="n"/>
-      <c r="T48" s="5" t="n"/>
-      <c r="U48" s="5" t="n"/>
-      <c r="V48" s="5" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n"/>
@@ -8370,9 +8154,6 @@
       <c r="Q49" s="5" t="n"/>
       <c r="R49" s="5" t="n"/>
       <c r="S49" s="5" t="n"/>
-      <c r="T49" s="5" t="n"/>
-      <c r="U49" s="5" t="n"/>
-      <c r="V49" s="5" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="n"/>
@@ -8394,9 +8175,6 @@
       <c r="Q50" s="5" t="n"/>
       <c r="R50" s="5" t="n"/>
       <c r="S50" s="5" t="n"/>
-      <c r="T50" s="5" t="n"/>
-      <c r="U50" s="5" t="n"/>
-      <c r="V50" s="5" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="n"/>
@@ -8418,9 +8196,6 @@
       <c r="Q51" s="5" t="n"/>
       <c r="R51" s="5" t="n"/>
       <c r="S51" s="5" t="n"/>
-      <c r="T51" s="5" t="n"/>
-      <c r="U51" s="5" t="n"/>
-      <c r="V51" s="5" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n"/>
@@ -8442,9 +8217,6 @@
       <c r="Q52" s="5" t="n"/>
       <c r="R52" s="5" t="n"/>
       <c r="S52" s="5" t="n"/>
-      <c r="T52" s="5" t="n"/>
-      <c r="U52" s="5" t="n"/>
-      <c r="V52" s="5" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="n"/>
@@ -8466,9 +8238,6 @@
       <c r="Q53" s="5" t="n"/>
       <c r="R53" s="5" t="n"/>
       <c r="S53" s="5" t="n"/>
-      <c r="T53" s="5" t="n"/>
-      <c r="U53" s="5" t="n"/>
-      <c r="V53" s="5" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n"/>
@@ -8490,9 +8259,6 @@
       <c r="Q54" s="5" t="n"/>
       <c r="R54" s="5" t="n"/>
       <c r="S54" s="5" t="n"/>
-      <c r="T54" s="5" t="n"/>
-      <c r="U54" s="5" t="n"/>
-      <c r="V54" s="5" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="n"/>
@@ -8514,9 +8280,6 @@
       <c r="Q55" s="5" t="n"/>
       <c r="R55" s="5" t="n"/>
       <c r="S55" s="5" t="n"/>
-      <c r="T55" s="5" t="n"/>
-      <c r="U55" s="5" t="n"/>
-      <c r="V55" s="5" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="n"/>
@@ -8538,9 +8301,6 @@
       <c r="Q56" s="5" t="n"/>
       <c r="R56" s="5" t="n"/>
       <c r="S56" s="5" t="n"/>
-      <c r="T56" s="5" t="n"/>
-      <c r="U56" s="5" t="n"/>
-      <c r="V56" s="5" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="n"/>
@@ -8562,9 +8322,6 @@
       <c r="Q57" s="5" t="n"/>
       <c r="R57" s="5" t="n"/>
       <c r="S57" s="5" t="n"/>
-      <c r="T57" s="5" t="n"/>
-      <c r="U57" s="5" t="n"/>
-      <c r="V57" s="5" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n"/>
@@ -8586,9 +8343,6 @@
       <c r="Q58" s="5" t="n"/>
       <c r="R58" s="5" t="n"/>
       <c r="S58" s="5" t="n"/>
-      <c r="T58" s="5" t="n"/>
-      <c r="U58" s="5" t="n"/>
-      <c r="V58" s="5" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="n"/>
@@ -8610,9 +8364,6 @@
       <c r="Q59" s="5" t="n"/>
       <c r="R59" s="5" t="n"/>
       <c r="S59" s="5" t="n"/>
-      <c r="T59" s="5" t="n"/>
-      <c r="U59" s="5" t="n"/>
-      <c r="V59" s="5" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="n"/>
@@ -8634,9 +8385,6 @@
       <c r="Q60" s="5" t="n"/>
       <c r="R60" s="5" t="n"/>
       <c r="S60" s="5" t="n"/>
-      <c r="T60" s="5" t="n"/>
-      <c r="U60" s="5" t="n"/>
-      <c r="V60" s="5" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="n"/>
@@ -8658,9 +8406,6 @@
       <c r="Q61" s="5" t="n"/>
       <c r="R61" s="5" t="n"/>
       <c r="S61" s="5" t="n"/>
-      <c r="T61" s="5" t="n"/>
-      <c r="U61" s="5" t="n"/>
-      <c r="V61" s="5" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="3" t="n"/>
@@ -8682,9 +8427,6 @@
       <c r="Q62" s="5" t="n"/>
       <c r="R62" s="5" t="n"/>
       <c r="S62" s="5" t="n"/>
-      <c r="T62" s="5" t="n"/>
-      <c r="U62" s="5" t="n"/>
-      <c r="V62" s="5" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="n"/>
@@ -8706,9 +8448,6 @@
       <c r="Q63" s="5" t="n"/>
       <c r="R63" s="5" t="n"/>
       <c r="S63" s="5" t="n"/>
-      <c r="T63" s="5" t="n"/>
-      <c r="U63" s="5" t="n"/>
-      <c r="V63" s="5" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="3" t="n"/>
@@ -8730,9 +8469,6 @@
       <c r="Q64" s="5" t="n"/>
       <c r="R64" s="5" t="n"/>
       <c r="S64" s="5" t="n"/>
-      <c r="T64" s="5" t="n"/>
-      <c r="U64" s="5" t="n"/>
-      <c r="V64" s="5" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="3" t="n"/>
@@ -8754,9 +8490,6 @@
       <c r="Q65" s="5" t="n"/>
       <c r="R65" s="5" t="n"/>
       <c r="S65" s="5" t="n"/>
-      <c r="T65" s="5" t="n"/>
-      <c r="U65" s="5" t="n"/>
-      <c r="V65" s="5" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="3" t="n"/>
@@ -8778,9 +8511,6 @@
       <c r="Q66" s="5" t="n"/>
       <c r="R66" s="5" t="n"/>
       <c r="S66" s="5" t="n"/>
-      <c r="T66" s="5" t="n"/>
-      <c r="U66" s="5" t="n"/>
-      <c r="V66" s="5" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="3" t="n"/>
@@ -8802,9 +8532,6 @@
       <c r="Q67" s="5" t="n"/>
       <c r="R67" s="5" t="n"/>
       <c r="S67" s="5" t="n"/>
-      <c r="T67" s="5" t="n"/>
-      <c r="U67" s="5" t="n"/>
-      <c r="V67" s="5" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="3" t="n"/>
@@ -8826,9 +8553,6 @@
       <c r="Q68" s="5" t="n"/>
       <c r="R68" s="5" t="n"/>
       <c r="S68" s="5" t="n"/>
-      <c r="T68" s="5" t="n"/>
-      <c r="U68" s="5" t="n"/>
-      <c r="V68" s="5" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="3" t="n"/>
@@ -8850,9 +8574,6 @@
       <c r="Q69" s="5" t="n"/>
       <c r="R69" s="5" t="n"/>
       <c r="S69" s="5" t="n"/>
-      <c r="T69" s="5" t="n"/>
-      <c r="U69" s="5" t="n"/>
-      <c r="V69" s="5" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="3" t="n"/>
@@ -8874,9 +8595,6 @@
       <c r="Q70" s="5" t="n"/>
       <c r="R70" s="5" t="n"/>
       <c r="S70" s="5" t="n"/>
-      <c r="T70" s="5" t="n"/>
-      <c r="U70" s="5" t="n"/>
-      <c r="V70" s="5" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="3" t="n"/>
@@ -8898,9 +8616,6 @@
       <c r="Q71" s="5" t="n"/>
       <c r="R71" s="5" t="n"/>
       <c r="S71" s="5" t="n"/>
-      <c r="T71" s="5" t="n"/>
-      <c r="U71" s="5" t="n"/>
-      <c r="V71" s="5" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="3" t="n"/>
@@ -8922,9 +8637,6 @@
       <c r="Q72" s="5" t="n"/>
       <c r="R72" s="5" t="n"/>
       <c r="S72" s="5" t="n"/>
-      <c r="T72" s="5" t="n"/>
-      <c r="U72" s="5" t="n"/>
-      <c r="V72" s="5" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="3" t="n"/>
@@ -8946,9 +8658,6 @@
       <c r="Q73" s="5" t="n"/>
       <c r="R73" s="5" t="n"/>
       <c r="S73" s="5" t="n"/>
-      <c r="T73" s="5" t="n"/>
-      <c r="U73" s="5" t="n"/>
-      <c r="V73" s="5" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="3" t="n"/>
@@ -8970,9 +8679,6 @@
       <c r="Q74" s="5" t="n"/>
       <c r="R74" s="5" t="n"/>
       <c r="S74" s="5" t="n"/>
-      <c r="T74" s="5" t="n"/>
-      <c r="U74" s="5" t="n"/>
-      <c r="V74" s="5" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="3" t="n"/>
@@ -8994,9 +8700,6 @@
       <c r="Q75" s="5" t="n"/>
       <c r="R75" s="5" t="n"/>
       <c r="S75" s="5" t="n"/>
-      <c r="T75" s="5" t="n"/>
-      <c r="U75" s="5" t="n"/>
-      <c r="V75" s="5" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="3" t="n"/>
@@ -9018,9 +8721,6 @@
       <c r="Q76" s="5" t="n"/>
       <c r="R76" s="5" t="n"/>
       <c r="S76" s="5" t="n"/>
-      <c r="T76" s="5" t="n"/>
-      <c r="U76" s="5" t="n"/>
-      <c r="V76" s="5" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="3" t="n"/>
@@ -9042,9 +8742,6 @@
       <c r="Q77" s="5" t="n"/>
       <c r="R77" s="5" t="n"/>
       <c r="S77" s="5" t="n"/>
-      <c r="T77" s="5" t="n"/>
-      <c r="U77" s="5" t="n"/>
-      <c r="V77" s="5" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="3" t="n"/>
@@ -9066,9 +8763,6 @@
       <c r="Q78" s="5" t="n"/>
       <c r="R78" s="5" t="n"/>
       <c r="S78" s="5" t="n"/>
-      <c r="T78" s="5" t="n"/>
-      <c r="U78" s="5" t="n"/>
-      <c r="V78" s="5" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="3" t="n"/>
@@ -9090,9 +8784,6 @@
       <c r="Q79" s="5" t="n"/>
       <c r="R79" s="5" t="n"/>
       <c r="S79" s="5" t="n"/>
-      <c r="T79" s="5" t="n"/>
-      <c r="U79" s="5" t="n"/>
-      <c r="V79" s="5" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="3" t="n"/>
@@ -9114,9 +8805,6 @@
       <c r="Q80" s="5" t="n"/>
       <c r="R80" s="5" t="n"/>
       <c r="S80" s="5" t="n"/>
-      <c r="T80" s="5" t="n"/>
-      <c r="U80" s="5" t="n"/>
-      <c r="V80" s="5" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="3" t="n"/>
@@ -9138,9 +8826,6 @@
       <c r="Q81" s="5" t="n"/>
       <c r="R81" s="5" t="n"/>
       <c r="S81" s="5" t="n"/>
-      <c r="T81" s="5" t="n"/>
-      <c r="U81" s="5" t="n"/>
-      <c r="V81" s="5" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="3" t="n"/>
@@ -9162,9 +8847,6 @@
       <c r="Q82" s="5" t="n"/>
       <c r="R82" s="5" t="n"/>
       <c r="S82" s="5" t="n"/>
-      <c r="T82" s="5" t="n"/>
-      <c r="U82" s="5" t="n"/>
-      <c r="V82" s="5" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="3" t="n"/>
@@ -9186,9 +8868,6 @@
       <c r="Q83" s="5" t="n"/>
       <c r="R83" s="5" t="n"/>
       <c r="S83" s="5" t="n"/>
-      <c r="T83" s="5" t="n"/>
-      <c r="U83" s="5" t="n"/>
-      <c r="V83" s="5" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="3" t="n"/>
@@ -9210,9 +8889,6 @@
       <c r="Q84" s="5" t="n"/>
       <c r="R84" s="5" t="n"/>
       <c r="S84" s="5" t="n"/>
-      <c r="T84" s="5" t="n"/>
-      <c r="U84" s="5" t="n"/>
-      <c r="V84" s="5" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="3" t="n"/>
@@ -9234,9 +8910,6 @@
       <c r="Q85" s="5" t="n"/>
       <c r="R85" s="5" t="n"/>
       <c r="S85" s="5" t="n"/>
-      <c r="T85" s="5" t="n"/>
-      <c r="U85" s="5" t="n"/>
-      <c r="V85" s="5" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="3" t="n"/>
@@ -9258,9 +8931,6 @@
       <c r="Q86" s="5" t="n"/>
       <c r="R86" s="5" t="n"/>
       <c r="S86" s="5" t="n"/>
-      <c r="T86" s="5" t="n"/>
-      <c r="U86" s="5" t="n"/>
-      <c r="V86" s="5" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="3" t="n"/>
@@ -9282,9 +8952,6 @@
       <c r="Q87" s="5" t="n"/>
       <c r="R87" s="5" t="n"/>
       <c r="S87" s="5" t="n"/>
-      <c r="T87" s="5" t="n"/>
-      <c r="U87" s="5" t="n"/>
-      <c r="V87" s="5" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="3" t="n"/>
@@ -9306,9 +8973,6 @@
       <c r="Q88" s="5" t="n"/>
       <c r="R88" s="5" t="n"/>
       <c r="S88" s="5" t="n"/>
-      <c r="T88" s="5" t="n"/>
-      <c r="U88" s="5" t="n"/>
-      <c r="V88" s="5" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="3" t="n"/>
@@ -9330,9 +8994,6 @@
       <c r="Q89" s="5" t="n"/>
       <c r="R89" s="5" t="n"/>
       <c r="S89" s="5" t="n"/>
-      <c r="T89" s="5" t="n"/>
-      <c r="U89" s="5" t="n"/>
-      <c r="V89" s="5" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="3" t="n"/>
@@ -9354,9 +9015,6 @@
       <c r="Q90" s="5" t="n"/>
       <c r="R90" s="5" t="n"/>
       <c r="S90" s="5" t="n"/>
-      <c r="T90" s="5" t="n"/>
-      <c r="U90" s="5" t="n"/>
-      <c r="V90" s="5" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="3" t="n"/>
@@ -9378,9 +9036,6 @@
       <c r="Q91" s="5" t="n"/>
       <c r="R91" s="5" t="n"/>
       <c r="S91" s="5" t="n"/>
-      <c r="T91" s="5" t="n"/>
-      <c r="U91" s="5" t="n"/>
-      <c r="V91" s="5" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="3" t="n"/>
@@ -9402,9 +9057,6 @@
       <c r="Q92" s="5" t="n"/>
       <c r="R92" s="5" t="n"/>
       <c r="S92" s="5" t="n"/>
-      <c r="T92" s="5" t="n"/>
-      <c r="U92" s="5" t="n"/>
-      <c r="V92" s="5" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="3" t="n"/>
@@ -9426,9 +9078,6 @@
       <c r="Q93" s="5" t="n"/>
       <c r="R93" s="5" t="n"/>
       <c r="S93" s="5" t="n"/>
-      <c r="T93" s="5" t="n"/>
-      <c r="U93" s="5" t="n"/>
-      <c r="V93" s="5" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="3" t="n"/>
@@ -9450,9 +9099,6 @@
       <c r="Q94" s="5" t="n"/>
       <c r="R94" s="5" t="n"/>
       <c r="S94" s="5" t="n"/>
-      <c r="T94" s="5" t="n"/>
-      <c r="U94" s="5" t="n"/>
-      <c r="V94" s="5" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="3" t="n"/>
@@ -9474,9 +9120,6 @@
       <c r="Q95" s="5" t="n"/>
       <c r="R95" s="5" t="n"/>
       <c r="S95" s="5" t="n"/>
-      <c r="T95" s="5" t="n"/>
-      <c r="U95" s="5" t="n"/>
-      <c r="V95" s="5" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="3" t="n"/>
@@ -9498,9 +9141,6 @@
       <c r="Q96" s="5" t="n"/>
       <c r="R96" s="5" t="n"/>
       <c r="S96" s="5" t="n"/>
-      <c r="T96" s="5" t="n"/>
-      <c r="U96" s="5" t="n"/>
-      <c r="V96" s="5" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="3" t="n"/>
@@ -9522,9 +9162,6 @@
       <c r="Q97" s="5" t="n"/>
       <c r="R97" s="5" t="n"/>
       <c r="S97" s="5" t="n"/>
-      <c r="T97" s="5" t="n"/>
-      <c r="U97" s="5" t="n"/>
-      <c r="V97" s="5" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="3" t="n"/>
@@ -9546,9 +9183,6 @@
       <c r="Q98" s="5" t="n"/>
       <c r="R98" s="5" t="n"/>
       <c r="S98" s="5" t="n"/>
-      <c r="T98" s="5" t="n"/>
-      <c r="U98" s="5" t="n"/>
-      <c r="V98" s="5" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="3" t="n"/>
@@ -9570,9 +9204,6 @@
       <c r="Q99" s="5" t="n"/>
       <c r="R99" s="5" t="n"/>
       <c r="S99" s="5" t="n"/>
-      <c r="T99" s="5" t="n"/>
-      <c r="U99" s="5" t="n"/>
-      <c r="V99" s="5" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="3" t="n"/>
@@ -9594,9 +9225,6 @@
       <c r="Q100" s="5" t="n"/>
       <c r="R100" s="5" t="n"/>
       <c r="S100" s="5" t="n"/>
-      <c r="T100" s="5" t="n"/>
-      <c r="U100" s="5" t="n"/>
-      <c r="V100" s="5" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="3" t="n"/>
@@ -9618,9 +9246,6 @@
       <c r="Q101" s="5" t="n"/>
       <c r="R101" s="5" t="n"/>
       <c r="S101" s="5" t="n"/>
-      <c r="T101" s="5" t="n"/>
-      <c r="U101" s="5" t="n"/>
-      <c r="V101" s="5" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="3" t="n"/>
@@ -9642,9 +9267,6 @@
       <c r="Q102" s="5" t="n"/>
       <c r="R102" s="5" t="n"/>
       <c r="S102" s="5" t="n"/>
-      <c r="T102" s="5" t="n"/>
-      <c r="U102" s="5" t="n"/>
-      <c r="V102" s="5" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="3" t="n"/>
@@ -9666,9 +9288,6 @@
       <c r="Q103" s="5" t="n"/>
       <c r="R103" s="5" t="n"/>
       <c r="S103" s="5" t="n"/>
-      <c r="T103" s="5" t="n"/>
-      <c r="U103" s="5" t="n"/>
-      <c r="V103" s="5" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="3" t="n"/>
@@ -9690,9 +9309,6 @@
       <c r="Q104" s="5" t="n"/>
       <c r="R104" s="5" t="n"/>
       <c r="S104" s="5" t="n"/>
-      <c r="T104" s="5" t="n"/>
-      <c r="U104" s="5" t="n"/>
-      <c r="V104" s="5" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="3" t="n"/>
@@ -9714,9 +9330,6 @@
       <c r="Q105" s="5" t="n"/>
       <c r="R105" s="5" t="n"/>
       <c r="S105" s="5" t="n"/>
-      <c r="T105" s="5" t="n"/>
-      <c r="U105" s="5" t="n"/>
-      <c r="V105" s="5" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="3" t="n"/>
@@ -9738,9 +9351,6 @@
       <c r="Q106" s="5" t="n"/>
       <c r="R106" s="5" t="n"/>
       <c r="S106" s="5" t="n"/>
-      <c r="T106" s="5" t="n"/>
-      <c r="U106" s="5" t="n"/>
-      <c r="V106" s="5" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="3" t="n"/>
@@ -9762,9 +9372,6 @@
       <c r="Q107" s="5" t="n"/>
       <c r="R107" s="5" t="n"/>
       <c r="S107" s="5" t="n"/>
-      <c r="T107" s="5" t="n"/>
-      <c r="U107" s="5" t="n"/>
-      <c r="V107" s="5" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="3" t="n"/>
@@ -9786,9 +9393,6 @@
       <c r="Q108" s="5" t="n"/>
       <c r="R108" s="5" t="n"/>
       <c r="S108" s="5" t="n"/>
-      <c r="T108" s="5" t="n"/>
-      <c r="U108" s="5" t="n"/>
-      <c r="V108" s="5" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="3" t="n"/>
@@ -9810,9 +9414,6 @@
       <c r="Q109" s="5" t="n"/>
       <c r="R109" s="5" t="n"/>
       <c r="S109" s="5" t="n"/>
-      <c r="T109" s="5" t="n"/>
-      <c r="U109" s="5" t="n"/>
-      <c r="V109" s="5" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="4">
@@ -9820,10 +9421,10 @@
     <dataValidation sqref="D9:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>TypeDefinitions!$W$2:$W$3</formula1>
     </dataValidation>
-    <dataValidation sqref="J9:J1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G9:G1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>TypeDefinitions!$X$2:$X$177</formula1>
     </dataValidation>
-    <dataValidation sqref="L9:L1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I9:I1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>TypeDefinitions!$Y$2:$Y$17</formula1>
     </dataValidation>
   </dataValidations>
@@ -60075,6 +59676,11 @@
           <t>Argentina</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>5A (Cool - Humid)</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
           <t>BREEAM</t>
@@ -60122,6 +59728,11 @@
           <t>Armenia</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>5B (Cool - Dry)</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
           <t>EDGE</t>
@@ -60169,6 +59780,11 @@
           <t>Aruba</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>5C (Cool - Marine)</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr">
         <is>
           <t>WELL</t>
@@ -60211,6 +59827,11 @@
           <t>Australia</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>6A (Cold - Humid)</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr">
         <is>
           <t>Other</t>
@@ -60251,6 +59872,11 @@
       <c r="C15" t="inlineStr">
         <is>
           <t>Austria</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>6B (Cold - Dry)</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">

</xml_diff>

<commit_message>
fix: cola general info
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -9613,23 +9613,23 @@
     <col width="48" customWidth="1" min="170" max="170"/>
     <col width="48" customWidth="1" min="171" max="171"/>
     <col width="49" customWidth="1" min="172" max="172"/>
-    <col width="52" customWidth="1" min="173" max="173"/>
-    <col width="49" customWidth="1" min="174" max="174"/>
-    <col width="49" customWidth="1" min="175" max="175"/>
-    <col width="49" customWidth="1" min="176" max="176"/>
-    <col width="49" customWidth="1" min="177" max="177"/>
-    <col width="49" customWidth="1" min="178" max="178"/>
-    <col width="49" customWidth="1" min="179" max="179"/>
-    <col width="49" customWidth="1" min="180" max="180"/>
-    <col width="49" customWidth="1" min="181" max="181"/>
-    <col width="49" customWidth="1" min="182" max="182"/>
-    <col width="49" customWidth="1" min="183" max="183"/>
-    <col width="49" customWidth="1" min="184" max="184"/>
-    <col width="49" customWidth="1" min="185" max="185"/>
-    <col width="48" customWidth="1" min="186" max="186"/>
-    <col width="49" customWidth="1" min="187" max="187"/>
-    <col width="49" customWidth="1" min="188" max="188"/>
-    <col width="50" customWidth="1" min="189" max="189"/>
+    <col width="51" customWidth="1" min="173" max="173"/>
+    <col width="48" customWidth="1" min="174" max="174"/>
+    <col width="48" customWidth="1" min="175" max="175"/>
+    <col width="48" customWidth="1" min="176" max="176"/>
+    <col width="48" customWidth="1" min="177" max="177"/>
+    <col width="48" customWidth="1" min="178" max="178"/>
+    <col width="48" customWidth="1" min="179" max="179"/>
+    <col width="48" customWidth="1" min="180" max="180"/>
+    <col width="48" customWidth="1" min="181" max="181"/>
+    <col width="48" customWidth="1" min="182" max="182"/>
+    <col width="48" customWidth="1" min="183" max="183"/>
+    <col width="48" customWidth="1" min="184" max="184"/>
+    <col width="48" customWidth="1" min="185" max="185"/>
+    <col width="47" customWidth="1" min="186" max="186"/>
+    <col width="48" customWidth="1" min="187" max="187"/>
+    <col width="48" customWidth="1" min="188" max="188"/>
+    <col width="49" customWidth="1" min="189" max="189"/>
     <col width="35" customWidth="1" min="190" max="190"/>
     <col width="32" customWidth="1" min="191" max="191"/>
     <col width="32" customWidth="1" min="192" max="192"/>
@@ -10648,87 +10648,87 @@
       </c>
       <c r="FQ1" s="1" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential (A1-A3)</t>
+          <t>Photochemical Ozone Creation Potential (A1-A3)</t>
         </is>
       </c>
       <c r="FR1" s="1" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential (A4)</t>
+          <t>Photochemical Ozone Creation Potential (A4)</t>
         </is>
       </c>
       <c r="FS1" s="1" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential (A5)</t>
+          <t>Photochemical Ozone Creation Potential (A5)</t>
         </is>
       </c>
       <c r="FT1" s="1" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential (B1)</t>
+          <t>Photochemical Ozone Creation Potential (B1)</t>
         </is>
       </c>
       <c r="FU1" s="1" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential (B2)</t>
+          <t>Photochemical Ozone Creation Potential (B2)</t>
         </is>
       </c>
       <c r="FV1" s="1" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential (B3)</t>
+          <t>Photochemical Ozone Creation Potential (B3)</t>
         </is>
       </c>
       <c r="FW1" s="1" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential (B4)</t>
+          <t>Photochemical Ozone Creation Potential (B4)</t>
         </is>
       </c>
       <c r="FX1" s="1" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential (B5)</t>
+          <t>Photochemical Ozone Creation Potential (B5)</t>
         </is>
       </c>
       <c r="FY1" s="1" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential (B6)</t>
+          <t>Photochemical Ozone Creation Potential (B6)</t>
         </is>
       </c>
       <c r="FZ1" s="1" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential (C1)</t>
+          <t>Photochemical Ozone Creation Potential (C1)</t>
         </is>
       </c>
       <c r="GA1" s="1" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential (C2)</t>
+          <t>Photochemical Ozone Creation Potential (C2)</t>
         </is>
       </c>
       <c r="GB1" s="1" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential (C3)</t>
+          <t>Photochemical Ozone Creation Potential (C3)</t>
         </is>
       </c>
       <c r="GC1" s="1" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential (C4)</t>
+          <t>Photochemical Ozone Creation Potential (C4)</t>
         </is>
       </c>
       <c r="GD1" s="1" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential (D)</t>
+          <t>Photochemical Ozone Creation Potential (D)</t>
         </is>
       </c>
       <c r="GE1" s="1" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential (D1)</t>
+          <t>Photochemical Ozone Creation Potential (D1)</t>
         </is>
       </c>
       <c r="GF1" s="1" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential (D2)</t>
+          <t>Photochemical Ozone Creation Potential (D2)</t>
         </is>
       </c>
       <c r="GG1" s="1" t="inlineStr">
         <is>
-          <t>Total Photochemical Ozone Formation Potential</t>
+          <t>Total Photochemical Ozone Creation Potential</t>
         </is>
       </c>
       <c r="GH1" s="1" t="inlineStr">
@@ -12360,87 +12360,87 @@
       </c>
       <c r="FQ2" s="10" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential for module A1-A3.</t>
+          <t>Photochemical Ozone Creation Potential for module A1-A3.</t>
         </is>
       </c>
       <c r="FR2" s="10" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential for module A4.</t>
+          <t>Photochemical Ozone Creation Potential for module A4.</t>
         </is>
       </c>
       <c r="FS2" s="10" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential for module A5.</t>
+          <t>Photochemical Ozone Creation Potential for module A5.</t>
         </is>
       </c>
       <c r="FT2" s="10" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential for module B1.</t>
+          <t>Photochemical Ozone Creation Potential for module B1.</t>
         </is>
       </c>
       <c r="FU2" s="10" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential for module B2.</t>
+          <t>Photochemical Ozone Creation Potential for module B2.</t>
         </is>
       </c>
       <c r="FV2" s="10" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential for module B3.</t>
+          <t>Photochemical Ozone Creation Potential for module B3.</t>
         </is>
       </c>
       <c r="FW2" s="10" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential for module B4.</t>
+          <t>Photochemical Ozone Creation Potential for module B4.</t>
         </is>
       </c>
       <c r="FX2" s="10" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential for module B5.</t>
+          <t>Photochemical Ozone Creation Potential for module B5.</t>
         </is>
       </c>
       <c r="FY2" s="10" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential for module B6.</t>
+          <t>Photochemical Ozone Creation Potential for module B6.</t>
         </is>
       </c>
       <c r="FZ2" s="10" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential for module C1.</t>
+          <t>Photochemical Ozone Creation Potential for module C1.</t>
         </is>
       </c>
       <c r="GA2" s="10" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential for module C2.</t>
+          <t>Photochemical Ozone Creation Potential for module C2.</t>
         </is>
       </c>
       <c r="GB2" s="10" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential for module C3.</t>
+          <t>Photochemical Ozone Creation Potential for module C3.</t>
         </is>
       </c>
       <c r="GC2" s="10" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential for module C4.</t>
+          <t>Photochemical Ozone Creation Potential for module C4.</t>
         </is>
       </c>
       <c r="GD2" s="10" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential for module D.</t>
+          <t>Photochemical Ozone Creation Potential for module D.</t>
         </is>
       </c>
       <c r="GE2" s="10" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential for module D1.</t>
+          <t>Photochemical Ozone Creation Potential for module D1.</t>
         </is>
       </c>
       <c r="GF2" s="10" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential for module D2.</t>
+          <t>Photochemical Ozone Creation Potential for module D2.</t>
         </is>
       </c>
       <c r="GG2" s="10" t="inlineStr">
         <is>
-          <t>Total Photochemical Ozone Formation Potential.</t>
+          <t>Total Photochemical Ozone Creation Potential.</t>
         </is>
       </c>
       <c r="GH2" s="10" t="inlineStr">
@@ -55184,7 +55184,7 @@
     <col width="50" customWidth="1" min="12" max="12"/>
     <col width="46" customWidth="1" min="13" max="13"/>
     <col width="43" customWidth="1" min="14" max="14"/>
-    <col width="44" customWidth="1" min="15" max="15"/>
+    <col width="43" customWidth="1" min="15" max="15"/>
     <col width="27" customWidth="1" min="16" max="16"/>
     <col width="44" customWidth="1" min="17" max="17"/>
     <col width="54" customWidth="1" min="18" max="18"/>
@@ -55269,7 +55269,7 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential</t>
+          <t>Photochemical Ozone Creation Potential</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
@@ -55391,7 +55391,7 @@
       </c>
       <c r="O2" s="10" t="inlineStr">
         <is>
-          <t>Photochemical Ozone Formation Potential.</t>
+          <t>Photochemical Ozone Creation Potential.</t>
         </is>
       </c>
       <c r="P2" s="10" t="inlineStr">

</xml_diff>

<commit_message>
feat: parse floor level
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -2466,27 +2466,27 @@
       <c r="J45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="inlineStr">
+      <c r="A46" t="inlineStr">
         <is>
           <t>Building</t>
         </is>
       </c>
-      <c r="B46" s="6" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>Building data (general)</t>
         </is>
       </c>
-      <c r="C46" s="6" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>Construction end date</t>
         </is>
       </c>
-      <c r="D46" s="6" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t>building_construction_end_date</t>
         </is>
       </c>
-      <c r="E46" s="6" t="inlineStr">
+      <c r="E46" t="inlineStr">
         <is>
           <t>The year/date building construction completed.</t>
         </is>
@@ -2498,9 +2498,9 @@
       </c>
       <c r="G46" s="3" t="inlineStr"/>
       <c r="H46" s="3" t="n"/>
-      <c r="I46" s="6" t="inlineStr">
-        <is>
-          <t>Required</t>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>Recommended</t>
         </is>
       </c>
       <c r="J46" s="5" t="inlineStr"/>
@@ -6493,7 +6493,7 @@
     <dataValidation sqref="J45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" operator="greaterThanOrEqual">
       <formula1>1900-01-01</formula1>
     </dataValidation>
-    <dataValidation sqref="J46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="date" operator="greaterThanOrEqual">
+    <dataValidation sqref="J46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" operator="greaterThanOrEqual">
       <formula1>1900-01-01</formula1>
     </dataValidation>
     <dataValidation sqref="J53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
feat: automatic wide to tall conversion
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -6672,7 +6672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S109"/>
+  <dimension ref="A1:T109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -6688,12 +6688,13 @@
     <col width="36" customWidth="1" min="11" max="11"/>
     <col width="31" customWidth="1" min="12" max="12"/>
     <col width="31" customWidth="1" min="13" max="13"/>
-    <col width="27" customWidth="1" min="14" max="14"/>
+    <col width="17" customWidth="1" min="14" max="14"/>
     <col width="27" customWidth="1" min="15" max="15"/>
-    <col width="26" customWidth="1" min="16" max="16"/>
-    <col width="30" customWidth="1" min="17" max="17"/>
-    <col width="25" customWidth="1" min="18" max="18"/>
-    <col width="15" customWidth="1" min="19" max="19"/>
+    <col width="27" customWidth="1" min="16" max="16"/>
+    <col width="26" customWidth="1" min="17" max="17"/>
+    <col width="30" customWidth="1" min="18" max="18"/>
+    <col width="25" customWidth="1" min="19" max="19"/>
+    <col width="15" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6764,30 +6765,35 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
+          <t>Service life</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>Material Quantity (m3)</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Material Quantity (m2)</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Material Quantity (m)</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Material Quantity (count)</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Material Weight (kg)</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Density</t>
         </is>
@@ -6859,32 +6865,37 @@
           <t>The URL of the specific Environmental Product Declaration (EPD) dataset used.</t>
         </is>
       </c>
-      <c r="N2" s="10" t="inlineStr">
+      <c r="N2" s="9" t="inlineStr">
+        <is>
+          <t>Declared reference service life.</t>
+        </is>
+      </c>
+      <c r="O2" s="10" t="inlineStr">
         <is>
           <t>The measured scalar amount (volume) of the custom material.</t>
         </is>
       </c>
-      <c r="O2" s="10" t="inlineStr">
+      <c r="P2" s="10" t="inlineStr">
         <is>
           <t>The measured scalar amount (area) of the custom material.</t>
         </is>
       </c>
-      <c r="P2" s="10" t="inlineStr">
+      <c r="Q2" s="10" t="inlineStr">
         <is>
           <t>The measured scalar amount (length) of the custom material.</t>
         </is>
       </c>
-      <c r="Q2" s="10" t="inlineStr">
+      <c r="R2" s="10" t="inlineStr">
         <is>
           <t>The measured scalar amount (count) of the custom material.</t>
         </is>
       </c>
-      <c r="R2" s="10" t="inlineStr">
+      <c r="S2" s="10" t="inlineStr">
         <is>
           <t>The absolute physical mass of the custom material.</t>
         </is>
       </c>
-      <c r="S2" s="10" t="inlineStr">
+      <c r="T2" s="10" t="inlineStr">
         <is>
           <t>The mass per unit volume of the custom material.</t>
         </is>
@@ -6982,6 +6993,11 @@
         </is>
       </c>
       <c r="S3" t="inlineStr">
+        <is>
+          <t>Decimal</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
         <is>
           <t>Decimal</t>
         </is>
@@ -7043,6 +7059,7 @@
       <c r="Q4" s="3" t="inlineStr"/>
       <c r="R4" s="3" t="inlineStr"/>
       <c r="S4" s="3" t="inlineStr"/>
+      <c r="T4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -7064,30 +7081,35 @@
       <c r="M5" s="3" t="n"/>
       <c r="N5" s="2" t="inlineStr">
         <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
           <t>m3</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>m2</t>
         </is>
       </c>
-      <c r="P5" s="2" t="inlineStr">
+      <c r="Q5" s="2" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="Q5" s="2" t="inlineStr">
+      <c r="R5" s="2" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="R5" s="2" t="inlineStr">
+      <c r="S5" s="2" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="S5" s="2" t="inlineStr">
+      <c r="T5" s="2" t="inlineStr">
         <is>
           <t>kg/m3</t>
         </is>
@@ -7159,32 +7181,37 @@
           <t>Optional</t>
         </is>
       </c>
-      <c r="N6" s="4" t="inlineStr">
+      <c r="N6" s="6" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="O6" s="4" t="inlineStr">
+      <c r="P6" s="4" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="P6" s="4" t="inlineStr">
+      <c r="Q6" s="4" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="Q6" s="4" t="inlineStr">
+      <c r="R6" s="4" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="R6" s="6" t="inlineStr">
+      <c r="S6" s="6" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="S6" s="4" t="inlineStr">
+      <c r="T6" s="4" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
@@ -7265,30 +7292,35 @@
       </c>
       <c r="N8" s="11" t="inlineStr">
         <is>
+          <t>lca_service_life</t>
+        </is>
+      </c>
+      <c r="O8" s="11" t="inlineStr">
+        <is>
           <t>custom_material_quantity_m3</t>
         </is>
       </c>
-      <c r="O8" s="11" t="inlineStr">
+      <c r="P8" s="11" t="inlineStr">
         <is>
           <t>custom_material_quantity_m2</t>
         </is>
       </c>
-      <c r="P8" s="11" t="inlineStr">
+      <c r="Q8" s="11" t="inlineStr">
         <is>
           <t>custom_material_quantity_m</t>
         </is>
       </c>
-      <c r="Q8" s="11" t="inlineStr">
+      <c r="R8" s="11" t="inlineStr">
         <is>
           <t>custom_material_quantity_count</t>
         </is>
       </c>
-      <c r="R8" s="11" t="inlineStr">
+      <c r="S8" s="11" t="inlineStr">
         <is>
           <t>custom_material_weight_kg</t>
         </is>
       </c>
-      <c r="S8" s="11" t="inlineStr">
+      <c r="T8" s="11" t="inlineStr">
         <is>
           <t>custom_material_density</t>
         </is>
@@ -7314,6 +7346,7 @@
       <c r="Q9" s="5" t="n"/>
       <c r="R9" s="5" t="n"/>
       <c r="S9" s="5" t="n"/>
+      <c r="T9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n"/>
@@ -7335,6 +7368,7 @@
       <c r="Q10" s="5" t="n"/>
       <c r="R10" s="5" t="n"/>
       <c r="S10" s="5" t="n"/>
+      <c r="T10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n"/>
@@ -7356,6 +7390,7 @@
       <c r="Q11" s="5" t="n"/>
       <c r="R11" s="5" t="n"/>
       <c r="S11" s="5" t="n"/>
+      <c r="T11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n"/>
@@ -7377,6 +7412,7 @@
       <c r="Q12" s="5" t="n"/>
       <c r="R12" s="5" t="n"/>
       <c r="S12" s="5" t="n"/>
+      <c r="T12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n"/>
@@ -7398,6 +7434,7 @@
       <c r="Q13" s="5" t="n"/>
       <c r="R13" s="5" t="n"/>
       <c r="S13" s="5" t="n"/>
+      <c r="T13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n"/>
@@ -7419,6 +7456,7 @@
       <c r="Q14" s="5" t="n"/>
       <c r="R14" s="5" t="n"/>
       <c r="S14" s="5" t="n"/>
+      <c r="T14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n"/>
@@ -7440,6 +7478,7 @@
       <c r="Q15" s="5" t="n"/>
       <c r="R15" s="5" t="n"/>
       <c r="S15" s="5" t="n"/>
+      <c r="T15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n"/>
@@ -7461,6 +7500,7 @@
       <c r="Q16" s="5" t="n"/>
       <c r="R16" s="5" t="n"/>
       <c r="S16" s="5" t="n"/>
+      <c r="T16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n"/>
@@ -7482,6 +7522,7 @@
       <c r="Q17" s="5" t="n"/>
       <c r="R17" s="5" t="n"/>
       <c r="S17" s="5" t="n"/>
+      <c r="T17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n"/>
@@ -7503,6 +7544,7 @@
       <c r="Q18" s="5" t="n"/>
       <c r="R18" s="5" t="n"/>
       <c r="S18" s="5" t="n"/>
+      <c r="T18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n"/>
@@ -7524,6 +7566,7 @@
       <c r="Q19" s="5" t="n"/>
       <c r="R19" s="5" t="n"/>
       <c r="S19" s="5" t="n"/>
+      <c r="T19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n"/>
@@ -7545,6 +7588,7 @@
       <c r="Q20" s="5" t="n"/>
       <c r="R20" s="5" t="n"/>
       <c r="S20" s="5" t="n"/>
+      <c r="T20" s="5" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n"/>
@@ -7566,6 +7610,7 @@
       <c r="Q21" s="5" t="n"/>
       <c r="R21" s="5" t="n"/>
       <c r="S21" s="5" t="n"/>
+      <c r="T21" s="5" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n"/>
@@ -7587,6 +7632,7 @@
       <c r="Q22" s="5" t="n"/>
       <c r="R22" s="5" t="n"/>
       <c r="S22" s="5" t="n"/>
+      <c r="T22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n"/>
@@ -7608,6 +7654,7 @@
       <c r="Q23" s="5" t="n"/>
       <c r="R23" s="5" t="n"/>
       <c r="S23" s="5" t="n"/>
+      <c r="T23" s="5" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n"/>
@@ -7629,6 +7676,7 @@
       <c r="Q24" s="5" t="n"/>
       <c r="R24" s="5" t="n"/>
       <c r="S24" s="5" t="n"/>
+      <c r="T24" s="5" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n"/>
@@ -7650,6 +7698,7 @@
       <c r="Q25" s="5" t="n"/>
       <c r="R25" s="5" t="n"/>
       <c r="S25" s="5" t="n"/>
+      <c r="T25" s="5" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n"/>
@@ -7671,6 +7720,7 @@
       <c r="Q26" s="5" t="n"/>
       <c r="R26" s="5" t="n"/>
       <c r="S26" s="5" t="n"/>
+      <c r="T26" s="5" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n"/>
@@ -7692,6 +7742,7 @@
       <c r="Q27" s="5" t="n"/>
       <c r="R27" s="5" t="n"/>
       <c r="S27" s="5" t="n"/>
+      <c r="T27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n"/>
@@ -7713,6 +7764,7 @@
       <c r="Q28" s="5" t="n"/>
       <c r="R28" s="5" t="n"/>
       <c r="S28" s="5" t="n"/>
+      <c r="T28" s="5" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n"/>
@@ -7734,6 +7786,7 @@
       <c r="Q29" s="5" t="n"/>
       <c r="R29" s="5" t="n"/>
       <c r="S29" s="5" t="n"/>
+      <c r="T29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n"/>
@@ -7755,6 +7808,7 @@
       <c r="Q30" s="5" t="n"/>
       <c r="R30" s="5" t="n"/>
       <c r="S30" s="5" t="n"/>
+      <c r="T30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n"/>
@@ -7776,6 +7830,7 @@
       <c r="Q31" s="5" t="n"/>
       <c r="R31" s="5" t="n"/>
       <c r="S31" s="5" t="n"/>
+      <c r="T31" s="5" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n"/>
@@ -7797,6 +7852,7 @@
       <c r="Q32" s="5" t="n"/>
       <c r="R32" s="5" t="n"/>
       <c r="S32" s="5" t="n"/>
+      <c r="T32" s="5" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n"/>
@@ -7818,6 +7874,7 @@
       <c r="Q33" s="5" t="n"/>
       <c r="R33" s="5" t="n"/>
       <c r="S33" s="5" t="n"/>
+      <c r="T33" s="5" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n"/>
@@ -7839,6 +7896,7 @@
       <c r="Q34" s="5" t="n"/>
       <c r="R34" s="5" t="n"/>
       <c r="S34" s="5" t="n"/>
+      <c r="T34" s="5" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n"/>
@@ -7860,6 +7918,7 @@
       <c r="Q35" s="5" t="n"/>
       <c r="R35" s="5" t="n"/>
       <c r="S35" s="5" t="n"/>
+      <c r="T35" s="5" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n"/>
@@ -7881,6 +7940,7 @@
       <c r="Q36" s="5" t="n"/>
       <c r="R36" s="5" t="n"/>
       <c r="S36" s="5" t="n"/>
+      <c r="T36" s="5" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n"/>
@@ -7902,6 +7962,7 @@
       <c r="Q37" s="5" t="n"/>
       <c r="R37" s="5" t="n"/>
       <c r="S37" s="5" t="n"/>
+      <c r="T37" s="5" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n"/>
@@ -7923,6 +7984,7 @@
       <c r="Q38" s="5" t="n"/>
       <c r="R38" s="5" t="n"/>
       <c r="S38" s="5" t="n"/>
+      <c r="T38" s="5" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n"/>
@@ -7944,6 +8006,7 @@
       <c r="Q39" s="5" t="n"/>
       <c r="R39" s="5" t="n"/>
       <c r="S39" s="5" t="n"/>
+      <c r="T39" s="5" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n"/>
@@ -7965,6 +8028,7 @@
       <c r="Q40" s="5" t="n"/>
       <c r="R40" s="5" t="n"/>
       <c r="S40" s="5" t="n"/>
+      <c r="T40" s="5" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n"/>
@@ -7986,6 +8050,7 @@
       <c r="Q41" s="5" t="n"/>
       <c r="R41" s="5" t="n"/>
       <c r="S41" s="5" t="n"/>
+      <c r="T41" s="5" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n"/>
@@ -8007,6 +8072,7 @@
       <c r="Q42" s="5" t="n"/>
       <c r="R42" s="5" t="n"/>
       <c r="S42" s="5" t="n"/>
+      <c r="T42" s="5" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n"/>
@@ -8028,6 +8094,7 @@
       <c r="Q43" s="5" t="n"/>
       <c r="R43" s="5" t="n"/>
       <c r="S43" s="5" t="n"/>
+      <c r="T43" s="5" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n"/>
@@ -8049,6 +8116,7 @@
       <c r="Q44" s="5" t="n"/>
       <c r="R44" s="5" t="n"/>
       <c r="S44" s="5" t="n"/>
+      <c r="T44" s="5" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="n"/>
@@ -8070,6 +8138,7 @@
       <c r="Q45" s="5" t="n"/>
       <c r="R45" s="5" t="n"/>
       <c r="S45" s="5" t="n"/>
+      <c r="T45" s="5" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n"/>
@@ -8091,6 +8160,7 @@
       <c r="Q46" s="5" t="n"/>
       <c r="R46" s="5" t="n"/>
       <c r="S46" s="5" t="n"/>
+      <c r="T46" s="5" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n"/>
@@ -8112,6 +8182,7 @@
       <c r="Q47" s="5" t="n"/>
       <c r="R47" s="5" t="n"/>
       <c r="S47" s="5" t="n"/>
+      <c r="T47" s="5" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n"/>
@@ -8133,6 +8204,7 @@
       <c r="Q48" s="5" t="n"/>
       <c r="R48" s="5" t="n"/>
       <c r="S48" s="5" t="n"/>
+      <c r="T48" s="5" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n"/>
@@ -8154,6 +8226,7 @@
       <c r="Q49" s="5" t="n"/>
       <c r="R49" s="5" t="n"/>
       <c r="S49" s="5" t="n"/>
+      <c r="T49" s="5" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="n"/>
@@ -8175,6 +8248,7 @@
       <c r="Q50" s="5" t="n"/>
       <c r="R50" s="5" t="n"/>
       <c r="S50" s="5" t="n"/>
+      <c r="T50" s="5" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="n"/>
@@ -8196,6 +8270,7 @@
       <c r="Q51" s="5" t="n"/>
       <c r="R51" s="5" t="n"/>
       <c r="S51" s="5" t="n"/>
+      <c r="T51" s="5" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n"/>
@@ -8217,6 +8292,7 @@
       <c r="Q52" s="5" t="n"/>
       <c r="R52" s="5" t="n"/>
       <c r="S52" s="5" t="n"/>
+      <c r="T52" s="5" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="n"/>
@@ -8238,6 +8314,7 @@
       <c r="Q53" s="5" t="n"/>
       <c r="R53" s="5" t="n"/>
       <c r="S53" s="5" t="n"/>
+      <c r="T53" s="5" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n"/>
@@ -8259,6 +8336,7 @@
       <c r="Q54" s="5" t="n"/>
       <c r="R54" s="5" t="n"/>
       <c r="S54" s="5" t="n"/>
+      <c r="T54" s="5" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="n"/>
@@ -8280,6 +8358,7 @@
       <c r="Q55" s="5" t="n"/>
       <c r="R55" s="5" t="n"/>
       <c r="S55" s="5" t="n"/>
+      <c r="T55" s="5" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="n"/>
@@ -8301,6 +8380,7 @@
       <c r="Q56" s="5" t="n"/>
       <c r="R56" s="5" t="n"/>
       <c r="S56" s="5" t="n"/>
+      <c r="T56" s="5" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="n"/>
@@ -8322,6 +8402,7 @@
       <c r="Q57" s="5" t="n"/>
       <c r="R57" s="5" t="n"/>
       <c r="S57" s="5" t="n"/>
+      <c r="T57" s="5" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n"/>
@@ -8343,6 +8424,7 @@
       <c r="Q58" s="5" t="n"/>
       <c r="R58" s="5" t="n"/>
       <c r="S58" s="5" t="n"/>
+      <c r="T58" s="5" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="n"/>
@@ -8364,6 +8446,7 @@
       <c r="Q59" s="5" t="n"/>
       <c r="R59" s="5" t="n"/>
       <c r="S59" s="5" t="n"/>
+      <c r="T59" s="5" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="n"/>
@@ -8385,6 +8468,7 @@
       <c r="Q60" s="5" t="n"/>
       <c r="R60" s="5" t="n"/>
       <c r="S60" s="5" t="n"/>
+      <c r="T60" s="5" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="n"/>
@@ -8406,6 +8490,7 @@
       <c r="Q61" s="5" t="n"/>
       <c r="R61" s="5" t="n"/>
       <c r="S61" s="5" t="n"/>
+      <c r="T61" s="5" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="3" t="n"/>
@@ -8427,6 +8512,7 @@
       <c r="Q62" s="5" t="n"/>
       <c r="R62" s="5" t="n"/>
       <c r="S62" s="5" t="n"/>
+      <c r="T62" s="5" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="n"/>
@@ -8448,6 +8534,7 @@
       <c r="Q63" s="5" t="n"/>
       <c r="R63" s="5" t="n"/>
       <c r="S63" s="5" t="n"/>
+      <c r="T63" s="5" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="3" t="n"/>
@@ -8469,6 +8556,7 @@
       <c r="Q64" s="5" t="n"/>
       <c r="R64" s="5" t="n"/>
       <c r="S64" s="5" t="n"/>
+      <c r="T64" s="5" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="3" t="n"/>
@@ -8490,6 +8578,7 @@
       <c r="Q65" s="5" t="n"/>
       <c r="R65" s="5" t="n"/>
       <c r="S65" s="5" t="n"/>
+      <c r="T65" s="5" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="3" t="n"/>
@@ -8511,6 +8600,7 @@
       <c r="Q66" s="5" t="n"/>
       <c r="R66" s="5" t="n"/>
       <c r="S66" s="5" t="n"/>
+      <c r="T66" s="5" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="3" t="n"/>
@@ -8532,6 +8622,7 @@
       <c r="Q67" s="5" t="n"/>
       <c r="R67" s="5" t="n"/>
       <c r="S67" s="5" t="n"/>
+      <c r="T67" s="5" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="3" t="n"/>
@@ -8553,6 +8644,7 @@
       <c r="Q68" s="5" t="n"/>
       <c r="R68" s="5" t="n"/>
       <c r="S68" s="5" t="n"/>
+      <c r="T68" s="5" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="3" t="n"/>
@@ -8574,6 +8666,7 @@
       <c r="Q69" s="5" t="n"/>
       <c r="R69" s="5" t="n"/>
       <c r="S69" s="5" t="n"/>
+      <c r="T69" s="5" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="3" t="n"/>
@@ -8595,6 +8688,7 @@
       <c r="Q70" s="5" t="n"/>
       <c r="R70" s="5" t="n"/>
       <c r="S70" s="5" t="n"/>
+      <c r="T70" s="5" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="3" t="n"/>
@@ -8616,6 +8710,7 @@
       <c r="Q71" s="5" t="n"/>
       <c r="R71" s="5" t="n"/>
       <c r="S71" s="5" t="n"/>
+      <c r="T71" s="5" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="3" t="n"/>
@@ -8637,6 +8732,7 @@
       <c r="Q72" s="5" t="n"/>
       <c r="R72" s="5" t="n"/>
       <c r="S72" s="5" t="n"/>
+      <c r="T72" s="5" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="3" t="n"/>
@@ -8658,6 +8754,7 @@
       <c r="Q73" s="5" t="n"/>
       <c r="R73" s="5" t="n"/>
       <c r="S73" s="5" t="n"/>
+      <c r="T73" s="5" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="3" t="n"/>
@@ -8679,6 +8776,7 @@
       <c r="Q74" s="5" t="n"/>
       <c r="R74" s="5" t="n"/>
       <c r="S74" s="5" t="n"/>
+      <c r="T74" s="5" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="3" t="n"/>
@@ -8700,6 +8798,7 @@
       <c r="Q75" s="5" t="n"/>
       <c r="R75" s="5" t="n"/>
       <c r="S75" s="5" t="n"/>
+      <c r="T75" s="5" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="3" t="n"/>
@@ -8721,6 +8820,7 @@
       <c r="Q76" s="5" t="n"/>
       <c r="R76" s="5" t="n"/>
       <c r="S76" s="5" t="n"/>
+      <c r="T76" s="5" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="3" t="n"/>
@@ -8742,6 +8842,7 @@
       <c r="Q77" s="5" t="n"/>
       <c r="R77" s="5" t="n"/>
       <c r="S77" s="5" t="n"/>
+      <c r="T77" s="5" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="3" t="n"/>
@@ -8763,6 +8864,7 @@
       <c r="Q78" s="5" t="n"/>
       <c r="R78" s="5" t="n"/>
       <c r="S78" s="5" t="n"/>
+      <c r="T78" s="5" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="3" t="n"/>
@@ -8784,6 +8886,7 @@
       <c r="Q79" s="5" t="n"/>
       <c r="R79" s="5" t="n"/>
       <c r="S79" s="5" t="n"/>
+      <c r="T79" s="5" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="3" t="n"/>
@@ -8805,6 +8908,7 @@
       <c r="Q80" s="5" t="n"/>
       <c r="R80" s="5" t="n"/>
       <c r="S80" s="5" t="n"/>
+      <c r="T80" s="5" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="3" t="n"/>
@@ -8826,6 +8930,7 @@
       <c r="Q81" s="5" t="n"/>
       <c r="R81" s="5" t="n"/>
       <c r="S81" s="5" t="n"/>
+      <c r="T81" s="5" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="3" t="n"/>
@@ -8847,6 +8952,7 @@
       <c r="Q82" s="5" t="n"/>
       <c r="R82" s="5" t="n"/>
       <c r="S82" s="5" t="n"/>
+      <c r="T82" s="5" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="3" t="n"/>
@@ -8868,6 +8974,7 @@
       <c r="Q83" s="5" t="n"/>
       <c r="R83" s="5" t="n"/>
       <c r="S83" s="5" t="n"/>
+      <c r="T83" s="5" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="3" t="n"/>
@@ -8889,6 +8996,7 @@
       <c r="Q84" s="5" t="n"/>
       <c r="R84" s="5" t="n"/>
       <c r="S84" s="5" t="n"/>
+      <c r="T84" s="5" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="3" t="n"/>
@@ -8910,6 +9018,7 @@
       <c r="Q85" s="5" t="n"/>
       <c r="R85" s="5" t="n"/>
       <c r="S85" s="5" t="n"/>
+      <c r="T85" s="5" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="3" t="n"/>
@@ -8931,6 +9040,7 @@
       <c r="Q86" s="5" t="n"/>
       <c r="R86" s="5" t="n"/>
       <c r="S86" s="5" t="n"/>
+      <c r="T86" s="5" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="3" t="n"/>
@@ -8952,6 +9062,7 @@
       <c r="Q87" s="5" t="n"/>
       <c r="R87" s="5" t="n"/>
       <c r="S87" s="5" t="n"/>
+      <c r="T87" s="5" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="3" t="n"/>
@@ -8973,6 +9084,7 @@
       <c r="Q88" s="5" t="n"/>
       <c r="R88" s="5" t="n"/>
       <c r="S88" s="5" t="n"/>
+      <c r="T88" s="5" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="3" t="n"/>
@@ -8994,6 +9106,7 @@
       <c r="Q89" s="5" t="n"/>
       <c r="R89" s="5" t="n"/>
       <c r="S89" s="5" t="n"/>
+      <c r="T89" s="5" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="3" t="n"/>
@@ -9015,6 +9128,7 @@
       <c r="Q90" s="5" t="n"/>
       <c r="R90" s="5" t="n"/>
       <c r="S90" s="5" t="n"/>
+      <c r="T90" s="5" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="3" t="n"/>
@@ -9036,6 +9150,7 @@
       <c r="Q91" s="5" t="n"/>
       <c r="R91" s="5" t="n"/>
       <c r="S91" s="5" t="n"/>
+      <c r="T91" s="5" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="3" t="n"/>
@@ -9057,6 +9172,7 @@
       <c r="Q92" s="5" t="n"/>
       <c r="R92" s="5" t="n"/>
       <c r="S92" s="5" t="n"/>
+      <c r="T92" s="5" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="3" t="n"/>
@@ -9078,6 +9194,7 @@
       <c r="Q93" s="5" t="n"/>
       <c r="R93" s="5" t="n"/>
       <c r="S93" s="5" t="n"/>
+      <c r="T93" s="5" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="3" t="n"/>
@@ -9099,6 +9216,7 @@
       <c r="Q94" s="5" t="n"/>
       <c r="R94" s="5" t="n"/>
       <c r="S94" s="5" t="n"/>
+      <c r="T94" s="5" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="3" t="n"/>
@@ -9120,6 +9238,7 @@
       <c r="Q95" s="5" t="n"/>
       <c r="R95" s="5" t="n"/>
       <c r="S95" s="5" t="n"/>
+      <c r="T95" s="5" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="3" t="n"/>
@@ -9141,6 +9260,7 @@
       <c r="Q96" s="5" t="n"/>
       <c r="R96" s="5" t="n"/>
       <c r="S96" s="5" t="n"/>
+      <c r="T96" s="5" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="3" t="n"/>
@@ -9162,6 +9282,7 @@
       <c r="Q97" s="5" t="n"/>
       <c r="R97" s="5" t="n"/>
       <c r="S97" s="5" t="n"/>
+      <c r="T97" s="5" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="3" t="n"/>
@@ -9183,6 +9304,7 @@
       <c r="Q98" s="5" t="n"/>
       <c r="R98" s="5" t="n"/>
       <c r="S98" s="5" t="n"/>
+      <c r="T98" s="5" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="3" t="n"/>
@@ -9204,6 +9326,7 @@
       <c r="Q99" s="5" t="n"/>
       <c r="R99" s="5" t="n"/>
       <c r="S99" s="5" t="n"/>
+      <c r="T99" s="5" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="3" t="n"/>
@@ -9225,6 +9348,7 @@
       <c r="Q100" s="5" t="n"/>
       <c r="R100" s="5" t="n"/>
       <c r="S100" s="5" t="n"/>
+      <c r="T100" s="5" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="3" t="n"/>
@@ -9246,6 +9370,7 @@
       <c r="Q101" s="5" t="n"/>
       <c r="R101" s="5" t="n"/>
       <c r="S101" s="5" t="n"/>
+      <c r="T101" s="5" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="3" t="n"/>
@@ -9267,6 +9392,7 @@
       <c r="Q102" s="5" t="n"/>
       <c r="R102" s="5" t="n"/>
       <c r="S102" s="5" t="n"/>
+      <c r="T102" s="5" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="3" t="n"/>
@@ -9288,6 +9414,7 @@
       <c r="Q103" s="5" t="n"/>
       <c r="R103" s="5" t="n"/>
       <c r="S103" s="5" t="n"/>
+      <c r="T103" s="5" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="3" t="n"/>
@@ -9309,6 +9436,7 @@
       <c r="Q104" s="5" t="n"/>
       <c r="R104" s="5" t="n"/>
       <c r="S104" s="5" t="n"/>
+      <c r="T104" s="5" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="3" t="n"/>
@@ -9330,6 +9458,7 @@
       <c r="Q105" s="5" t="n"/>
       <c r="R105" s="5" t="n"/>
       <c r="S105" s="5" t="n"/>
+      <c r="T105" s="5" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="3" t="n"/>
@@ -9351,6 +9480,7 @@
       <c r="Q106" s="5" t="n"/>
       <c r="R106" s="5" t="n"/>
       <c r="S106" s="5" t="n"/>
+      <c r="T106" s="5" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="3" t="n"/>
@@ -9372,6 +9502,7 @@
       <c r="Q107" s="5" t="n"/>
       <c r="R107" s="5" t="n"/>
       <c r="S107" s="5" t="n"/>
+      <c r="T107" s="5" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="3" t="n"/>
@@ -9393,6 +9524,7 @@
       <c r="Q108" s="5" t="n"/>
       <c r="R108" s="5" t="n"/>
       <c r="S108" s="5" t="n"/>
+      <c r="T108" s="5" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="3" t="n"/>
@@ -9414,6 +9546,7 @@
       <c r="Q109" s="5" t="n"/>
       <c r="R109" s="5" t="n"/>
       <c r="S109" s="5" t="n"/>
+      <c r="T109" s="5" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="4">

</xml_diff>